<commit_message>
Tighten teardown claims to what the reviews show
An independent check found no wrong numbers or quotes, but some text said
more than the evidence: five-whys citations that didn't support every part
of their step, hypotheses shown as root-cause facts, and review shares
presented as support load. Root causes are now labelled likely, citations
match their reviews, and the impact copy says it assumes tickets mirror
reviews.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1yWPAzLJJuCYqF9DpXqGJ
</commit_message>
<xml_diff>
--- a/interview-demos/yesmadam-contact-drivers/Contact-Driver-Teardown.xlsx
+++ b/interview-demos/yesmadam-contact-drivers/Contact-Driver-Teardown.xlsx
@@ -65310,12 +65310,12 @@
     <row r="39">
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>rude_behaviour</t>
+          <t>hygiene</t>
         </is>
       </c>
       <c r="C39" s="27" t="inlineStr">
         <is>
-          <t>Rude behaviour</t>
+          <t>Hygiene</t>
         </is>
       </c>
       <c r="D39" s="21">
@@ -65330,12 +65330,12 @@
     <row r="40">
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>hygiene</t>
+          <t>safety_or_theft</t>
         </is>
       </c>
       <c r="C40" s="27" t="inlineStr">
         <is>
-          <t>Hygiene</t>
+          <t>Safety, privacy or theft</t>
         </is>
       </c>
       <c r="D40" s="21">
@@ -65350,12 +65350,12 @@
     <row r="41">
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>safety_or_theft</t>
+          <t>rude_behaviour</t>
         </is>
       </c>
       <c r="C41" s="27" t="inlineStr">
         <is>
-          <t>Safety, privacy or theft</t>
+          <t>Rude behaviour</t>
         </is>
       </c>
       <c r="D41" s="21">
@@ -65576,7 +65576,7 @@
       </c>
       <c r="C9" s="33" t="inlineStr">
         <is>
-          <t>Accepting a job does not lock the professional in. Some ask the customer to cancel instead, so the drop is logged as a customer cancellation (#127, #219, #362).</t>
+          <t>Accepting a job does not lock the professional in: some call and ask the customer to cancel instead (#127, #219, #362).</t>
         </is>
       </c>
       <c r="D9" s="34" t="n"/>
@@ -65733,7 +65733,7 @@
       </c>
       <c r="C21" s="33" t="inlineStr">
         <is>
-          <t>It reads as a scam, not a sell-out, because it is pushed to everyone without saying how many slots exist (#48, #77).</t>
+          <t>It reads as a scam, not a sell-out: customers call it 'fake' and 'bluffing', and nothing tells them how few slots there were (#48, #77, #121).</t>
         </is>
       </c>
       <c r="D21" s="34" t="n"/>
@@ -65790,7 +65790,7 @@
       </c>
       <c r="C24" s="37" t="inlineStr">
         <is>
-          <t>Offers and prices are built to attract, not to be honoured: a tiny flash offer pushed to everyone, and compulsory fees shown only at checkout.</t>
+          <t>Offers and prices are built to attract, not to be honoured: a flash offer that sells out in minutes is pushed to everyone, and compulsory fees show up only at checkout.</t>
         </is>
       </c>
     </row>
@@ -65852,7 +65852,7 @@
       </c>
       <c r="C31" s="33" t="inlineStr">
         <is>
-          <t>The professional lacked the skill for that service: burnt skin after waxing, ruined brows, half-done work (#41, #152, #191).</t>
+          <t>The professional lacked the skill for that service: burnt skin after waxing, ruined brows (#41, #152, #191).</t>
         </is>
       </c>
       <c r="D31" s="34" t="n"/>
@@ -65890,7 +65890,7 @@
       </c>
       <c r="C33" s="33" t="inlineStr">
         <is>
-          <t>Professionals rush the job ('in too much hurry', a facial done in 30 minutes), likely because back-to-back slots leave no slack (#50, #264, #351).</t>
+          <t>Professionals rush the job: 'in too much hurry', a facial done in 30 minutes (#50, #264, #351).</t>
         </is>
       </c>
       <c r="D33" s="34" t="n"/>
@@ -65909,7 +65909,7 @@
       </c>
       <c r="C34" s="33" t="inlineStr">
         <is>
-          <t>When something goes wrong, the answer is a coupon, not a call-back or care for the injury: a ₹400 coupon for a burnt hand (#41, #104, #217).</t>
+          <t>When something goes wrong, there is no real follow-up: a ₹400 coupon for a burnt hand, no reply to photos of a burn, a promised refund that never came (#41, #217, #104).</t>
         </is>
       </c>
       <c r="D34" s="34" t="n"/>
@@ -66840,7 +66840,7 @@
       </c>
       <c r="C5" s="32" t="inlineStr">
         <is>
-          <t>Customers who write reviews are mostly unhappy: 45% of the 500 most recent App Store reviews are 1★, against a 4.73★ store average.</t>
+          <t>Customers who write reviews are mostly unhappy: 58% of the 500 most recent App Store reviews are complaints and 45% are 1★, against a 4.73★ store average.</t>
         </is>
       </c>
     </row>
@@ -66895,7 +66895,7 @@
       </c>
       <c r="C11" s="32" t="inlineStr">
         <is>
-          <t>Offers and prices are built to attract, not to be honoured: a tiny flash offer pushed to everyone, and compulsory fees shown only at checkout.</t>
+          <t>Offers and prices are built to attract, not to be honoured: a flash offer that sells out in minutes is pushed to everyone, and compulsory fees show up only at checkout.</t>
         </is>
       </c>
     </row>

</xml_diff>